<commit_message>
fix: bare except → typed except + date check in add_row() for create_excel, create_pertanian, update_crypto, update_emas, update_harga, update_pertanian, precompute_analysis, proses_keuangan, validate_data
</commit_message>
<xml_diff>
--- a/data/crypto_monitor.xlsx
+++ b/data/crypto_monitor.xlsx
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V11"/>
+  <dimension ref="A1:V12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1412,6 +1412,80 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>O:0 H:0 L:0 C:0</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1778.96</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="I12" t="n">
+        <v>81.63</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>-0.2</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="n">
+        <v>8.779999999999999</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>NETRAL ⚪</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>